<commit_message>
collected enough data for step 2; wound down max thread size; made ANSI safe
</commit_message>
<xml_diff>
--- a/ci-cd-merge-resolver/repoCollector/datasets/Ant-Media-Server.xlsx
+++ b/ci-cd-merge-resolver/repoCollector/datasets/Ant-Media-Server.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>mergeCommit</t>
   </si>
@@ -44,13 +44,28 @@
     <t>isMultiModule</t>
   </si>
   <si>
+    <t>50607679762370f9dbddc306dbd23f8c18ae6705</t>
+  </si>
+  <si>
+    <t>c0c17460ea78f0485c37a3d0d3ffc2dd61ee27ec</t>
+  </si>
+  <si>
+    <t>4e1610905d024d5e2e6c1373e714e45435ae46f2</t>
+  </si>
+  <si>
     <t>af67326e6f3a26cafb268b1e8a413b7746108897</t>
   </si>
   <si>
-    <t>50607679762370f9dbddc306dbd23f8c18ae6705</t>
-  </si>
-  <si>
     <t>5e4f804865e1bfeb30713f42589e45c1171c800f</t>
+  </si>
+  <si>
+    <t>442ea9bc4b40466a924a7631b6be90caf5034815</t>
+  </si>
+  <si>
+    <t>8eba176315f0eeac59fa67d42890f5fe4d0c6388</t>
+  </si>
+  <si>
+    <t>c1a62fd392cdf1004887531904574cf7979127e3</t>
   </si>
 </sst>
 </file>
@@ -95,7 +110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -141,7 +156,7 @@
         <v>12</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>95.0</v>
+        <v>197.0</v>
       </c>
       <c r="E2" t="n" s="0">
         <v>1.0</v>
@@ -156,9 +171,73 @@
         <v>1</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>20.95800018310547</v>
+        <v>440.8090515136719</v>
       </c>
       <c r="J2" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D3" t="n" s="0">
+        <v>197.0</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="G3" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="H3" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n" s="0">
+        <v>446.4670104980469</v>
+      </c>
+      <c r="J3" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="D4" t="n" s="0">
+        <v>200.0</v>
+      </c>
+      <c r="E4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="G4" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="H4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n" s="0">
+        <v>501.3299865722656</v>
+      </c>
+      <c r="J4" t="b" s="0">
         <v>0</v>
       </c>
     </row>

</xml_diff>